<commit_message>
fix(accounting): upload shows existing codes as skipped; fix template dropdowns
</commit_message>
<xml_diff>
--- a/frontend/public/templates/SmartAppt_COAUpload_Template.xlsx
+++ b/frontend/public/templates/SmartAppt_COAUpload_Template.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart of Accounts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lookups" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -91,7 +92,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002563EB"/>
+        <fgColor rgb="001D4ED8"/>
       </patternFill>
     </fill>
     <fill>
@@ -158,13 +159,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -539,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -548,7 +549,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -557,7 +558,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SmartAppt – Chart of Accounts Upload Template  |  Blue = Required  |  Grey = Optional  |  Do not modify column headers (Row 2)  |  Date format: YYYY-MM-DD</t>
+          <t>SmartAppt – COA Upload Template  |  Blue header = Required  |  Grey header = Optional  |  Date format: YYYY-MM-DD  |  Do not edit rows 1–5</t>
         </is>
       </c>
     </row>
@@ -3109,19 +3110,1225 @@
       <c r="I200" s="8" t="n"/>
       <c r="J200" s="8" t="n"/>
     </row>
+    <row r="201" ht="17" customHeight="1">
+      <c r="A201" s="8" t="n"/>
+      <c r="B201" s="8" t="n"/>
+      <c r="C201" s="8" t="n"/>
+      <c r="D201" s="8" t="n"/>
+      <c r="E201" s="8" t="n"/>
+      <c r="F201" s="8" t="n"/>
+      <c r="G201" s="8" t="n"/>
+      <c r="H201" s="8" t="n"/>
+      <c r="I201" s="8" t="n"/>
+      <c r="J201" s="8" t="n"/>
+    </row>
+    <row r="202" ht="17" customHeight="1">
+      <c r="A202" s="8" t="n"/>
+      <c r="B202" s="8" t="n"/>
+      <c r="C202" s="8" t="n"/>
+      <c r="D202" s="8" t="n"/>
+      <c r="E202" s="8" t="n"/>
+      <c r="F202" s="8" t="n"/>
+      <c r="G202" s="8" t="n"/>
+      <c r="H202" s="8" t="n"/>
+      <c r="I202" s="8" t="n"/>
+      <c r="J202" s="8" t="n"/>
+    </row>
+    <row r="203" ht="17" customHeight="1">
+      <c r="A203" s="8" t="n"/>
+      <c r="B203" s="8" t="n"/>
+      <c r="C203" s="8" t="n"/>
+      <c r="D203" s="8" t="n"/>
+      <c r="E203" s="8" t="n"/>
+      <c r="F203" s="8" t="n"/>
+      <c r="G203" s="8" t="n"/>
+      <c r="H203" s="8" t="n"/>
+      <c r="I203" s="8" t="n"/>
+      <c r="J203" s="8" t="n"/>
+    </row>
+    <row r="204" ht="17" customHeight="1">
+      <c r="A204" s="8" t="n"/>
+      <c r="B204" s="8" t="n"/>
+      <c r="C204" s="8" t="n"/>
+      <c r="D204" s="8" t="n"/>
+      <c r="E204" s="8" t="n"/>
+      <c r="F204" s="8" t="n"/>
+      <c r="G204" s="8" t="n"/>
+      <c r="H204" s="8" t="n"/>
+      <c r="I204" s="8" t="n"/>
+      <c r="J204" s="8" t="n"/>
+    </row>
+    <row r="205" ht="17" customHeight="1">
+      <c r="A205" s="8" t="n"/>
+      <c r="B205" s="8" t="n"/>
+      <c r="C205" s="8" t="n"/>
+      <c r="D205" s="8" t="n"/>
+      <c r="E205" s="8" t="n"/>
+      <c r="F205" s="8" t="n"/>
+      <c r="G205" s="8" t="n"/>
+      <c r="H205" s="8" t="n"/>
+      <c r="I205" s="8" t="n"/>
+      <c r="J205" s="8" t="n"/>
+    </row>
+    <row r="206" ht="17" customHeight="1">
+      <c r="A206" s="8" t="n"/>
+      <c r="B206" s="8" t="n"/>
+      <c r="C206" s="8" t="n"/>
+      <c r="D206" s="8" t="n"/>
+      <c r="E206" s="8" t="n"/>
+      <c r="F206" s="8" t="n"/>
+      <c r="G206" s="8" t="n"/>
+      <c r="H206" s="8" t="n"/>
+      <c r="I206" s="8" t="n"/>
+      <c r="J206" s="8" t="n"/>
+    </row>
+    <row r="207" ht="17" customHeight="1">
+      <c r="A207" s="8" t="n"/>
+      <c r="B207" s="8" t="n"/>
+      <c r="C207" s="8" t="n"/>
+      <c r="D207" s="8" t="n"/>
+      <c r="E207" s="8" t="n"/>
+      <c r="F207" s="8" t="n"/>
+      <c r="G207" s="8" t="n"/>
+      <c r="H207" s="8" t="n"/>
+      <c r="I207" s="8" t="n"/>
+      <c r="J207" s="8" t="n"/>
+    </row>
+    <row r="208" ht="17" customHeight="1">
+      <c r="A208" s="8" t="n"/>
+      <c r="B208" s="8" t="n"/>
+      <c r="C208" s="8" t="n"/>
+      <c r="D208" s="8" t="n"/>
+      <c r="E208" s="8" t="n"/>
+      <c r="F208" s="8" t="n"/>
+      <c r="G208" s="8" t="n"/>
+      <c r="H208" s="8" t="n"/>
+      <c r="I208" s="8" t="n"/>
+      <c r="J208" s="8" t="n"/>
+    </row>
+    <row r="209" ht="17" customHeight="1">
+      <c r="A209" s="8" t="n"/>
+      <c r="B209" s="8" t="n"/>
+      <c r="C209" s="8" t="n"/>
+      <c r="D209" s="8" t="n"/>
+      <c r="E209" s="8" t="n"/>
+      <c r="F209" s="8" t="n"/>
+      <c r="G209" s="8" t="n"/>
+      <c r="H209" s="8" t="n"/>
+      <c r="I209" s="8" t="n"/>
+      <c r="J209" s="8" t="n"/>
+    </row>
+    <row r="210" ht="17" customHeight="1">
+      <c r="A210" s="8" t="n"/>
+      <c r="B210" s="8" t="n"/>
+      <c r="C210" s="8" t="n"/>
+      <c r="D210" s="8" t="n"/>
+      <c r="E210" s="8" t="n"/>
+      <c r="F210" s="8" t="n"/>
+      <c r="G210" s="8" t="n"/>
+      <c r="H210" s="8" t="n"/>
+      <c r="I210" s="8" t="n"/>
+      <c r="J210" s="8" t="n"/>
+    </row>
+    <row r="211" ht="17" customHeight="1">
+      <c r="A211" s="8" t="n"/>
+      <c r="B211" s="8" t="n"/>
+      <c r="C211" s="8" t="n"/>
+      <c r="D211" s="8" t="n"/>
+      <c r="E211" s="8" t="n"/>
+      <c r="F211" s="8" t="n"/>
+      <c r="G211" s="8" t="n"/>
+      <c r="H211" s="8" t="n"/>
+      <c r="I211" s="8" t="n"/>
+      <c r="J211" s="8" t="n"/>
+    </row>
+    <row r="212" ht="17" customHeight="1">
+      <c r="A212" s="8" t="n"/>
+      <c r="B212" s="8" t="n"/>
+      <c r="C212" s="8" t="n"/>
+      <c r="D212" s="8" t="n"/>
+      <c r="E212" s="8" t="n"/>
+      <c r="F212" s="8" t="n"/>
+      <c r="G212" s="8" t="n"/>
+      <c r="H212" s="8" t="n"/>
+      <c r="I212" s="8" t="n"/>
+      <c r="J212" s="8" t="n"/>
+    </row>
+    <row r="213" ht="17" customHeight="1">
+      <c r="A213" s="8" t="n"/>
+      <c r="B213" s="8" t="n"/>
+      <c r="C213" s="8" t="n"/>
+      <c r="D213" s="8" t="n"/>
+      <c r="E213" s="8" t="n"/>
+      <c r="F213" s="8" t="n"/>
+      <c r="G213" s="8" t="n"/>
+      <c r="H213" s="8" t="n"/>
+      <c r="I213" s="8" t="n"/>
+      <c r="J213" s="8" t="n"/>
+    </row>
+    <row r="214" ht="17" customHeight="1">
+      <c r="A214" s="8" t="n"/>
+      <c r="B214" s="8" t="n"/>
+      <c r="C214" s="8" t="n"/>
+      <c r="D214" s="8" t="n"/>
+      <c r="E214" s="8" t="n"/>
+      <c r="F214" s="8" t="n"/>
+      <c r="G214" s="8" t="n"/>
+      <c r="H214" s="8" t="n"/>
+      <c r="I214" s="8" t="n"/>
+      <c r="J214" s="8" t="n"/>
+    </row>
+    <row r="215" ht="17" customHeight="1">
+      <c r="A215" s="8" t="n"/>
+      <c r="B215" s="8" t="n"/>
+      <c r="C215" s="8" t="n"/>
+      <c r="D215" s="8" t="n"/>
+      <c r="E215" s="8" t="n"/>
+      <c r="F215" s="8" t="n"/>
+      <c r="G215" s="8" t="n"/>
+      <c r="H215" s="8" t="n"/>
+      <c r="I215" s="8" t="n"/>
+      <c r="J215" s="8" t="n"/>
+    </row>
+    <row r="216" ht="17" customHeight="1">
+      <c r="A216" s="8" t="n"/>
+      <c r="B216" s="8" t="n"/>
+      <c r="C216" s="8" t="n"/>
+      <c r="D216" s="8" t="n"/>
+      <c r="E216" s="8" t="n"/>
+      <c r="F216" s="8" t="n"/>
+      <c r="G216" s="8" t="n"/>
+      <c r="H216" s="8" t="n"/>
+      <c r="I216" s="8" t="n"/>
+      <c r="J216" s="8" t="n"/>
+    </row>
+    <row r="217" ht="17" customHeight="1">
+      <c r="A217" s="8" t="n"/>
+      <c r="B217" s="8" t="n"/>
+      <c r="C217" s="8" t="n"/>
+      <c r="D217" s="8" t="n"/>
+      <c r="E217" s="8" t="n"/>
+      <c r="F217" s="8" t="n"/>
+      <c r="G217" s="8" t="n"/>
+      <c r="H217" s="8" t="n"/>
+      <c r="I217" s="8" t="n"/>
+      <c r="J217" s="8" t="n"/>
+    </row>
+    <row r="218" ht="17" customHeight="1">
+      <c r="A218" s="8" t="n"/>
+      <c r="B218" s="8" t="n"/>
+      <c r="C218" s="8" t="n"/>
+      <c r="D218" s="8" t="n"/>
+      <c r="E218" s="8" t="n"/>
+      <c r="F218" s="8" t="n"/>
+      <c r="G218" s="8" t="n"/>
+      <c r="H218" s="8" t="n"/>
+      <c r="I218" s="8" t="n"/>
+      <c r="J218" s="8" t="n"/>
+    </row>
+    <row r="219" ht="17" customHeight="1">
+      <c r="A219" s="8" t="n"/>
+      <c r="B219" s="8" t="n"/>
+      <c r="C219" s="8" t="n"/>
+      <c r="D219" s="8" t="n"/>
+      <c r="E219" s="8" t="n"/>
+      <c r="F219" s="8" t="n"/>
+      <c r="G219" s="8" t="n"/>
+      <c r="H219" s="8" t="n"/>
+      <c r="I219" s="8" t="n"/>
+      <c r="J219" s="8" t="n"/>
+    </row>
+    <row r="220" ht="17" customHeight="1">
+      <c r="A220" s="8" t="n"/>
+      <c r="B220" s="8" t="n"/>
+      <c r="C220" s="8" t="n"/>
+      <c r="D220" s="8" t="n"/>
+      <c r="E220" s="8" t="n"/>
+      <c r="F220" s="8" t="n"/>
+      <c r="G220" s="8" t="n"/>
+      <c r="H220" s="8" t="n"/>
+      <c r="I220" s="8" t="n"/>
+      <c r="J220" s="8" t="n"/>
+    </row>
+    <row r="221" ht="17" customHeight="1">
+      <c r="A221" s="8" t="n"/>
+      <c r="B221" s="8" t="n"/>
+      <c r="C221" s="8" t="n"/>
+      <c r="D221" s="8" t="n"/>
+      <c r="E221" s="8" t="n"/>
+      <c r="F221" s="8" t="n"/>
+      <c r="G221" s="8" t="n"/>
+      <c r="H221" s="8" t="n"/>
+      <c r="I221" s="8" t="n"/>
+      <c r="J221" s="8" t="n"/>
+    </row>
+    <row r="222" ht="17" customHeight="1">
+      <c r="A222" s="8" t="n"/>
+      <c r="B222" s="8" t="n"/>
+      <c r="C222" s="8" t="n"/>
+      <c r="D222" s="8" t="n"/>
+      <c r="E222" s="8" t="n"/>
+      <c r="F222" s="8" t="n"/>
+      <c r="G222" s="8" t="n"/>
+      <c r="H222" s="8" t="n"/>
+      <c r="I222" s="8" t="n"/>
+      <c r="J222" s="8" t="n"/>
+    </row>
+    <row r="223" ht="17" customHeight="1">
+      <c r="A223" s="8" t="n"/>
+      <c r="B223" s="8" t="n"/>
+      <c r="C223" s="8" t="n"/>
+      <c r="D223" s="8" t="n"/>
+      <c r="E223" s="8" t="n"/>
+      <c r="F223" s="8" t="n"/>
+      <c r="G223" s="8" t="n"/>
+      <c r="H223" s="8" t="n"/>
+      <c r="I223" s="8" t="n"/>
+      <c r="J223" s="8" t="n"/>
+    </row>
+    <row r="224" ht="17" customHeight="1">
+      <c r="A224" s="8" t="n"/>
+      <c r="B224" s="8" t="n"/>
+      <c r="C224" s="8" t="n"/>
+      <c r="D224" s="8" t="n"/>
+      <c r="E224" s="8" t="n"/>
+      <c r="F224" s="8" t="n"/>
+      <c r="G224" s="8" t="n"/>
+      <c r="H224" s="8" t="n"/>
+      <c r="I224" s="8" t="n"/>
+      <c r="J224" s="8" t="n"/>
+    </row>
+    <row r="225" ht="17" customHeight="1">
+      <c r="A225" s="8" t="n"/>
+      <c r="B225" s="8" t="n"/>
+      <c r="C225" s="8" t="n"/>
+      <c r="D225" s="8" t="n"/>
+      <c r="E225" s="8" t="n"/>
+      <c r="F225" s="8" t="n"/>
+      <c r="G225" s="8" t="n"/>
+      <c r="H225" s="8" t="n"/>
+      <c r="I225" s="8" t="n"/>
+      <c r="J225" s="8" t="n"/>
+    </row>
+    <row r="226" ht="17" customHeight="1">
+      <c r="A226" s="8" t="n"/>
+      <c r="B226" s="8" t="n"/>
+      <c r="C226" s="8" t="n"/>
+      <c r="D226" s="8" t="n"/>
+      <c r="E226" s="8" t="n"/>
+      <c r="F226" s="8" t="n"/>
+      <c r="G226" s="8" t="n"/>
+      <c r="H226" s="8" t="n"/>
+      <c r="I226" s="8" t="n"/>
+      <c r="J226" s="8" t="n"/>
+    </row>
+    <row r="227" ht="17" customHeight="1">
+      <c r="A227" s="8" t="n"/>
+      <c r="B227" s="8" t="n"/>
+      <c r="C227" s="8" t="n"/>
+      <c r="D227" s="8" t="n"/>
+      <c r="E227" s="8" t="n"/>
+      <c r="F227" s="8" t="n"/>
+      <c r="G227" s="8" t="n"/>
+      <c r="H227" s="8" t="n"/>
+      <c r="I227" s="8" t="n"/>
+      <c r="J227" s="8" t="n"/>
+    </row>
+    <row r="228" ht="17" customHeight="1">
+      <c r="A228" s="8" t="n"/>
+      <c r="B228" s="8" t="n"/>
+      <c r="C228" s="8" t="n"/>
+      <c r="D228" s="8" t="n"/>
+      <c r="E228" s="8" t="n"/>
+      <c r="F228" s="8" t="n"/>
+      <c r="G228" s="8" t="n"/>
+      <c r="H228" s="8" t="n"/>
+      <c r="I228" s="8" t="n"/>
+      <c r="J228" s="8" t="n"/>
+    </row>
+    <row r="229" ht="17" customHeight="1">
+      <c r="A229" s="8" t="n"/>
+      <c r="B229" s="8" t="n"/>
+      <c r="C229" s="8" t="n"/>
+      <c r="D229" s="8" t="n"/>
+      <c r="E229" s="8" t="n"/>
+      <c r="F229" s="8" t="n"/>
+      <c r="G229" s="8" t="n"/>
+      <c r="H229" s="8" t="n"/>
+      <c r="I229" s="8" t="n"/>
+      <c r="J229" s="8" t="n"/>
+    </row>
+    <row r="230" ht="17" customHeight="1">
+      <c r="A230" s="8" t="n"/>
+      <c r="B230" s="8" t="n"/>
+      <c r="C230" s="8" t="n"/>
+      <c r="D230" s="8" t="n"/>
+      <c r="E230" s="8" t="n"/>
+      <c r="F230" s="8" t="n"/>
+      <c r="G230" s="8" t="n"/>
+      <c r="H230" s="8" t="n"/>
+      <c r="I230" s="8" t="n"/>
+      <c r="J230" s="8" t="n"/>
+    </row>
+    <row r="231" ht="17" customHeight="1">
+      <c r="A231" s="8" t="n"/>
+      <c r="B231" s="8" t="n"/>
+      <c r="C231" s="8" t="n"/>
+      <c r="D231" s="8" t="n"/>
+      <c r="E231" s="8" t="n"/>
+      <c r="F231" s="8" t="n"/>
+      <c r="G231" s="8" t="n"/>
+      <c r="H231" s="8" t="n"/>
+      <c r="I231" s="8" t="n"/>
+      <c r="J231" s="8" t="n"/>
+    </row>
+    <row r="232" ht="17" customHeight="1">
+      <c r="A232" s="8" t="n"/>
+      <c r="B232" s="8" t="n"/>
+      <c r="C232" s="8" t="n"/>
+      <c r="D232" s="8" t="n"/>
+      <c r="E232" s="8" t="n"/>
+      <c r="F232" s="8" t="n"/>
+      <c r="G232" s="8" t="n"/>
+      <c r="H232" s="8" t="n"/>
+      <c r="I232" s="8" t="n"/>
+      <c r="J232" s="8" t="n"/>
+    </row>
+    <row r="233" ht="17" customHeight="1">
+      <c r="A233" s="8" t="n"/>
+      <c r="B233" s="8" t="n"/>
+      <c r="C233" s="8" t="n"/>
+      <c r="D233" s="8" t="n"/>
+      <c r="E233" s="8" t="n"/>
+      <c r="F233" s="8" t="n"/>
+      <c r="G233" s="8" t="n"/>
+      <c r="H233" s="8" t="n"/>
+      <c r="I233" s="8" t="n"/>
+      <c r="J233" s="8" t="n"/>
+    </row>
+    <row r="234" ht="17" customHeight="1">
+      <c r="A234" s="8" t="n"/>
+      <c r="B234" s="8" t="n"/>
+      <c r="C234" s="8" t="n"/>
+      <c r="D234" s="8" t="n"/>
+      <c r="E234" s="8" t="n"/>
+      <c r="F234" s="8" t="n"/>
+      <c r="G234" s="8" t="n"/>
+      <c r="H234" s="8" t="n"/>
+      <c r="I234" s="8" t="n"/>
+      <c r="J234" s="8" t="n"/>
+    </row>
+    <row r="235" ht="17" customHeight="1">
+      <c r="A235" s="8" t="n"/>
+      <c r="B235" s="8" t="n"/>
+      <c r="C235" s="8" t="n"/>
+      <c r="D235" s="8" t="n"/>
+      <c r="E235" s="8" t="n"/>
+      <c r="F235" s="8" t="n"/>
+      <c r="G235" s="8" t="n"/>
+      <c r="H235" s="8" t="n"/>
+      <c r="I235" s="8" t="n"/>
+      <c r="J235" s="8" t="n"/>
+    </row>
+    <row r="236" ht="17" customHeight="1">
+      <c r="A236" s="8" t="n"/>
+      <c r="B236" s="8" t="n"/>
+      <c r="C236" s="8" t="n"/>
+      <c r="D236" s="8" t="n"/>
+      <c r="E236" s="8" t="n"/>
+      <c r="F236" s="8" t="n"/>
+      <c r="G236" s="8" t="n"/>
+      <c r="H236" s="8" t="n"/>
+      <c r="I236" s="8" t="n"/>
+      <c r="J236" s="8" t="n"/>
+    </row>
+    <row r="237" ht="17" customHeight="1">
+      <c r="A237" s="8" t="n"/>
+      <c r="B237" s="8" t="n"/>
+      <c r="C237" s="8" t="n"/>
+      <c r="D237" s="8" t="n"/>
+      <c r="E237" s="8" t="n"/>
+      <c r="F237" s="8" t="n"/>
+      <c r="G237" s="8" t="n"/>
+      <c r="H237" s="8" t="n"/>
+      <c r="I237" s="8" t="n"/>
+      <c r="J237" s="8" t="n"/>
+    </row>
+    <row r="238" ht="17" customHeight="1">
+      <c r="A238" s="8" t="n"/>
+      <c r="B238" s="8" t="n"/>
+      <c r="C238" s="8" t="n"/>
+      <c r="D238" s="8" t="n"/>
+      <c r="E238" s="8" t="n"/>
+      <c r="F238" s="8" t="n"/>
+      <c r="G238" s="8" t="n"/>
+      <c r="H238" s="8" t="n"/>
+      <c r="I238" s="8" t="n"/>
+      <c r="J238" s="8" t="n"/>
+    </row>
+    <row r="239" ht="17" customHeight="1">
+      <c r="A239" s="8" t="n"/>
+      <c r="B239" s="8" t="n"/>
+      <c r="C239" s="8" t="n"/>
+      <c r="D239" s="8" t="n"/>
+      <c r="E239" s="8" t="n"/>
+      <c r="F239" s="8" t="n"/>
+      <c r="G239" s="8" t="n"/>
+      <c r="H239" s="8" t="n"/>
+      <c r="I239" s="8" t="n"/>
+      <c r="J239" s="8" t="n"/>
+    </row>
+    <row r="240" ht="17" customHeight="1">
+      <c r="A240" s="8" t="n"/>
+      <c r="B240" s="8" t="n"/>
+      <c r="C240" s="8" t="n"/>
+      <c r="D240" s="8" t="n"/>
+      <c r="E240" s="8" t="n"/>
+      <c r="F240" s="8" t="n"/>
+      <c r="G240" s="8" t="n"/>
+      <c r="H240" s="8" t="n"/>
+      <c r="I240" s="8" t="n"/>
+      <c r="J240" s="8" t="n"/>
+    </row>
+    <row r="241" ht="17" customHeight="1">
+      <c r="A241" s="8" t="n"/>
+      <c r="B241" s="8" t="n"/>
+      <c r="C241" s="8" t="n"/>
+      <c r="D241" s="8" t="n"/>
+      <c r="E241" s="8" t="n"/>
+      <c r="F241" s="8" t="n"/>
+      <c r="G241" s="8" t="n"/>
+      <c r="H241" s="8" t="n"/>
+      <c r="I241" s="8" t="n"/>
+      <c r="J241" s="8" t="n"/>
+    </row>
+    <row r="242" ht="17" customHeight="1">
+      <c r="A242" s="8" t="n"/>
+      <c r="B242" s="8" t="n"/>
+      <c r="C242" s="8" t="n"/>
+      <c r="D242" s="8" t="n"/>
+      <c r="E242" s="8" t="n"/>
+      <c r="F242" s="8" t="n"/>
+      <c r="G242" s="8" t="n"/>
+      <c r="H242" s="8" t="n"/>
+      <c r="I242" s="8" t="n"/>
+      <c r="J242" s="8" t="n"/>
+    </row>
+    <row r="243" ht="17" customHeight="1">
+      <c r="A243" s="8" t="n"/>
+      <c r="B243" s="8" t="n"/>
+      <c r="C243" s="8" t="n"/>
+      <c r="D243" s="8" t="n"/>
+      <c r="E243" s="8" t="n"/>
+      <c r="F243" s="8" t="n"/>
+      <c r="G243" s="8" t="n"/>
+      <c r="H243" s="8" t="n"/>
+      <c r="I243" s="8" t="n"/>
+      <c r="J243" s="8" t="n"/>
+    </row>
+    <row r="244" ht="17" customHeight="1">
+      <c r="A244" s="8" t="n"/>
+      <c r="B244" s="8" t="n"/>
+      <c r="C244" s="8" t="n"/>
+      <c r="D244" s="8" t="n"/>
+      <c r="E244" s="8" t="n"/>
+      <c r="F244" s="8" t="n"/>
+      <c r="G244" s="8" t="n"/>
+      <c r="H244" s="8" t="n"/>
+      <c r="I244" s="8" t="n"/>
+      <c r="J244" s="8" t="n"/>
+    </row>
+    <row r="245" ht="17" customHeight="1">
+      <c r="A245" s="8" t="n"/>
+      <c r="B245" s="8" t="n"/>
+      <c r="C245" s="8" t="n"/>
+      <c r="D245" s="8" t="n"/>
+      <c r="E245" s="8" t="n"/>
+      <c r="F245" s="8" t="n"/>
+      <c r="G245" s="8" t="n"/>
+      <c r="H245" s="8" t="n"/>
+      <c r="I245" s="8" t="n"/>
+      <c r="J245" s="8" t="n"/>
+    </row>
+    <row r="246" ht="17" customHeight="1">
+      <c r="A246" s="8" t="n"/>
+      <c r="B246" s="8" t="n"/>
+      <c r="C246" s="8" t="n"/>
+      <c r="D246" s="8" t="n"/>
+      <c r="E246" s="8" t="n"/>
+      <c r="F246" s="8" t="n"/>
+      <c r="G246" s="8" t="n"/>
+      <c r="H246" s="8" t="n"/>
+      <c r="I246" s="8" t="n"/>
+      <c r="J246" s="8" t="n"/>
+    </row>
+    <row r="247" ht="17" customHeight="1">
+      <c r="A247" s="8" t="n"/>
+      <c r="B247" s="8" t="n"/>
+      <c r="C247" s="8" t="n"/>
+      <c r="D247" s="8" t="n"/>
+      <c r="E247" s="8" t="n"/>
+      <c r="F247" s="8" t="n"/>
+      <c r="G247" s="8" t="n"/>
+      <c r="H247" s="8" t="n"/>
+      <c r="I247" s="8" t="n"/>
+      <c r="J247" s="8" t="n"/>
+    </row>
+    <row r="248" ht="17" customHeight="1">
+      <c r="A248" s="8" t="n"/>
+      <c r="B248" s="8" t="n"/>
+      <c r="C248" s="8" t="n"/>
+      <c r="D248" s="8" t="n"/>
+      <c r="E248" s="8" t="n"/>
+      <c r="F248" s="8" t="n"/>
+      <c r="G248" s="8" t="n"/>
+      <c r="H248" s="8" t="n"/>
+      <c r="I248" s="8" t="n"/>
+      <c r="J248" s="8" t="n"/>
+    </row>
+    <row r="249" ht="17" customHeight="1">
+      <c r="A249" s="8" t="n"/>
+      <c r="B249" s="8" t="n"/>
+      <c r="C249" s="8" t="n"/>
+      <c r="D249" s="8" t="n"/>
+      <c r="E249" s="8" t="n"/>
+      <c r="F249" s="8" t="n"/>
+      <c r="G249" s="8" t="n"/>
+      <c r="H249" s="8" t="n"/>
+      <c r="I249" s="8" t="n"/>
+      <c r="J249" s="8" t="n"/>
+    </row>
+    <row r="250" ht="17" customHeight="1">
+      <c r="A250" s="8" t="n"/>
+      <c r="B250" s="8" t="n"/>
+      <c r="C250" s="8" t="n"/>
+      <c r="D250" s="8" t="n"/>
+      <c r="E250" s="8" t="n"/>
+      <c r="F250" s="8" t="n"/>
+      <c r="G250" s="8" t="n"/>
+      <c r="H250" s="8" t="n"/>
+      <c r="I250" s="8" t="n"/>
+      <c r="J250" s="8" t="n"/>
+    </row>
+    <row r="251" ht="17" customHeight="1">
+      <c r="A251" s="8" t="n"/>
+      <c r="B251" s="8" t="n"/>
+      <c r="C251" s="8" t="n"/>
+      <c r="D251" s="8" t="n"/>
+      <c r="E251" s="8" t="n"/>
+      <c r="F251" s="8" t="n"/>
+      <c r="G251" s="8" t="n"/>
+      <c r="H251" s="8" t="n"/>
+      <c r="I251" s="8" t="n"/>
+      <c r="J251" s="8" t="n"/>
+    </row>
+    <row r="252" ht="17" customHeight="1">
+      <c r="A252" s="8" t="n"/>
+      <c r="B252" s="8" t="n"/>
+      <c r="C252" s="8" t="n"/>
+      <c r="D252" s="8" t="n"/>
+      <c r="E252" s="8" t="n"/>
+      <c r="F252" s="8" t="n"/>
+      <c r="G252" s="8" t="n"/>
+      <c r="H252" s="8" t="n"/>
+      <c r="I252" s="8" t="n"/>
+      <c r="J252" s="8" t="n"/>
+    </row>
+    <row r="253" ht="17" customHeight="1">
+      <c r="A253" s="8" t="n"/>
+      <c r="B253" s="8" t="n"/>
+      <c r="C253" s="8" t="n"/>
+      <c r="D253" s="8" t="n"/>
+      <c r="E253" s="8" t="n"/>
+      <c r="F253" s="8" t="n"/>
+      <c r="G253" s="8" t="n"/>
+      <c r="H253" s="8" t="n"/>
+      <c r="I253" s="8" t="n"/>
+      <c r="J253" s="8" t="n"/>
+    </row>
+    <row r="254" ht="17" customHeight="1">
+      <c r="A254" s="8" t="n"/>
+      <c r="B254" s="8" t="n"/>
+      <c r="C254" s="8" t="n"/>
+      <c r="D254" s="8" t="n"/>
+      <c r="E254" s="8" t="n"/>
+      <c r="F254" s="8" t="n"/>
+      <c r="G254" s="8" t="n"/>
+      <c r="H254" s="8" t="n"/>
+      <c r="I254" s="8" t="n"/>
+      <c r="J254" s="8" t="n"/>
+    </row>
+    <row r="255" ht="17" customHeight="1">
+      <c r="A255" s="8" t="n"/>
+      <c r="B255" s="8" t="n"/>
+      <c r="C255" s="8" t="n"/>
+      <c r="D255" s="8" t="n"/>
+      <c r="E255" s="8" t="n"/>
+      <c r="F255" s="8" t="n"/>
+      <c r="G255" s="8" t="n"/>
+      <c r="H255" s="8" t="n"/>
+      <c r="I255" s="8" t="n"/>
+      <c r="J255" s="8" t="n"/>
+    </row>
+    <row r="256" ht="17" customHeight="1">
+      <c r="A256" s="8" t="n"/>
+      <c r="B256" s="8" t="n"/>
+      <c r="C256" s="8" t="n"/>
+      <c r="D256" s="8" t="n"/>
+      <c r="E256" s="8" t="n"/>
+      <c r="F256" s="8" t="n"/>
+      <c r="G256" s="8" t="n"/>
+      <c r="H256" s="8" t="n"/>
+      <c r="I256" s="8" t="n"/>
+      <c r="J256" s="8" t="n"/>
+    </row>
+    <row r="257" ht="17" customHeight="1">
+      <c r="A257" s="8" t="n"/>
+      <c r="B257" s="8" t="n"/>
+      <c r="C257" s="8" t="n"/>
+      <c r="D257" s="8" t="n"/>
+      <c r="E257" s="8" t="n"/>
+      <c r="F257" s="8" t="n"/>
+      <c r="G257" s="8" t="n"/>
+      <c r="H257" s="8" t="n"/>
+      <c r="I257" s="8" t="n"/>
+      <c r="J257" s="8" t="n"/>
+    </row>
+    <row r="258" ht="17" customHeight="1">
+      <c r="A258" s="8" t="n"/>
+      <c r="B258" s="8" t="n"/>
+      <c r="C258" s="8" t="n"/>
+      <c r="D258" s="8" t="n"/>
+      <c r="E258" s="8" t="n"/>
+      <c r="F258" s="8" t="n"/>
+      <c r="G258" s="8" t="n"/>
+      <c r="H258" s="8" t="n"/>
+      <c r="I258" s="8" t="n"/>
+      <c r="J258" s="8" t="n"/>
+    </row>
+    <row r="259" ht="17" customHeight="1">
+      <c r="A259" s="8" t="n"/>
+      <c r="B259" s="8" t="n"/>
+      <c r="C259" s="8" t="n"/>
+      <c r="D259" s="8" t="n"/>
+      <c r="E259" s="8" t="n"/>
+      <c r="F259" s="8" t="n"/>
+      <c r="G259" s="8" t="n"/>
+      <c r="H259" s="8" t="n"/>
+      <c r="I259" s="8" t="n"/>
+      <c r="J259" s="8" t="n"/>
+    </row>
+    <row r="260" ht="17" customHeight="1">
+      <c r="A260" s="8" t="n"/>
+      <c r="B260" s="8" t="n"/>
+      <c r="C260" s="8" t="n"/>
+      <c r="D260" s="8" t="n"/>
+      <c r="E260" s="8" t="n"/>
+      <c r="F260" s="8" t="n"/>
+      <c r="G260" s="8" t="n"/>
+      <c r="H260" s="8" t="n"/>
+      <c r="I260" s="8" t="n"/>
+      <c r="J260" s="8" t="n"/>
+    </row>
+    <row r="261" ht="17" customHeight="1">
+      <c r="A261" s="8" t="n"/>
+      <c r="B261" s="8" t="n"/>
+      <c r="C261" s="8" t="n"/>
+      <c r="D261" s="8" t="n"/>
+      <c r="E261" s="8" t="n"/>
+      <c r="F261" s="8" t="n"/>
+      <c r="G261" s="8" t="n"/>
+      <c r="H261" s="8" t="n"/>
+      <c r="I261" s="8" t="n"/>
+      <c r="J261" s="8" t="n"/>
+    </row>
+    <row r="262" ht="17" customHeight="1">
+      <c r="A262" s="8" t="n"/>
+      <c r="B262" s="8" t="n"/>
+      <c r="C262" s="8" t="n"/>
+      <c r="D262" s="8" t="n"/>
+      <c r="E262" s="8" t="n"/>
+      <c r="F262" s="8" t="n"/>
+      <c r="G262" s="8" t="n"/>
+      <c r="H262" s="8" t="n"/>
+      <c r="I262" s="8" t="n"/>
+      <c r="J262" s="8" t="n"/>
+    </row>
+    <row r="263" ht="17" customHeight="1">
+      <c r="A263" s="8" t="n"/>
+      <c r="B263" s="8" t="n"/>
+      <c r="C263" s="8" t="n"/>
+      <c r="D263" s="8" t="n"/>
+      <c r="E263" s="8" t="n"/>
+      <c r="F263" s="8" t="n"/>
+      <c r="G263" s="8" t="n"/>
+      <c r="H263" s="8" t="n"/>
+      <c r="I263" s="8" t="n"/>
+      <c r="J263" s="8" t="n"/>
+    </row>
+    <row r="264" ht="17" customHeight="1">
+      <c r="A264" s="8" t="n"/>
+      <c r="B264" s="8" t="n"/>
+      <c r="C264" s="8" t="n"/>
+      <c r="D264" s="8" t="n"/>
+      <c r="E264" s="8" t="n"/>
+      <c r="F264" s="8" t="n"/>
+      <c r="G264" s="8" t="n"/>
+      <c r="H264" s="8" t="n"/>
+      <c r="I264" s="8" t="n"/>
+      <c r="J264" s="8" t="n"/>
+    </row>
+    <row r="265" ht="17" customHeight="1">
+      <c r="A265" s="8" t="n"/>
+      <c r="B265" s="8" t="n"/>
+      <c r="C265" s="8" t="n"/>
+      <c r="D265" s="8" t="n"/>
+      <c r="E265" s="8" t="n"/>
+      <c r="F265" s="8" t="n"/>
+      <c r="G265" s="8" t="n"/>
+      <c r="H265" s="8" t="n"/>
+      <c r="I265" s="8" t="n"/>
+      <c r="J265" s="8" t="n"/>
+    </row>
+    <row r="266" ht="17" customHeight="1">
+      <c r="A266" s="8" t="n"/>
+      <c r="B266" s="8" t="n"/>
+      <c r="C266" s="8" t="n"/>
+      <c r="D266" s="8" t="n"/>
+      <c r="E266" s="8" t="n"/>
+      <c r="F266" s="8" t="n"/>
+      <c r="G266" s="8" t="n"/>
+      <c r="H266" s="8" t="n"/>
+      <c r="I266" s="8" t="n"/>
+      <c r="J266" s="8" t="n"/>
+    </row>
+    <row r="267" ht="17" customHeight="1">
+      <c r="A267" s="8" t="n"/>
+      <c r="B267" s="8" t="n"/>
+      <c r="C267" s="8" t="n"/>
+      <c r="D267" s="8" t="n"/>
+      <c r="E267" s="8" t="n"/>
+      <c r="F267" s="8" t="n"/>
+      <c r="G267" s="8" t="n"/>
+      <c r="H267" s="8" t="n"/>
+      <c r="I267" s="8" t="n"/>
+      <c r="J267" s="8" t="n"/>
+    </row>
+    <row r="268" ht="17" customHeight="1">
+      <c r="A268" s="8" t="n"/>
+      <c r="B268" s="8" t="n"/>
+      <c r="C268" s="8" t="n"/>
+      <c r="D268" s="8" t="n"/>
+      <c r="E268" s="8" t="n"/>
+      <c r="F268" s="8" t="n"/>
+      <c r="G268" s="8" t="n"/>
+      <c r="H268" s="8" t="n"/>
+      <c r="I268" s="8" t="n"/>
+      <c r="J268" s="8" t="n"/>
+    </row>
+    <row r="269" ht="17" customHeight="1">
+      <c r="A269" s="8" t="n"/>
+      <c r="B269" s="8" t="n"/>
+      <c r="C269" s="8" t="n"/>
+      <c r="D269" s="8" t="n"/>
+      <c r="E269" s="8" t="n"/>
+      <c r="F269" s="8" t="n"/>
+      <c r="G269" s="8" t="n"/>
+      <c r="H269" s="8" t="n"/>
+      <c r="I269" s="8" t="n"/>
+      <c r="J269" s="8" t="n"/>
+    </row>
+    <row r="270" ht="17" customHeight="1">
+      <c r="A270" s="8" t="n"/>
+      <c r="B270" s="8" t="n"/>
+      <c r="C270" s="8" t="n"/>
+      <c r="D270" s="8" t="n"/>
+      <c r="E270" s="8" t="n"/>
+      <c r="F270" s="8" t="n"/>
+      <c r="G270" s="8" t="n"/>
+      <c r="H270" s="8" t="n"/>
+      <c r="I270" s="8" t="n"/>
+      <c r="J270" s="8" t="n"/>
+    </row>
+    <row r="271" ht="17" customHeight="1">
+      <c r="A271" s="8" t="n"/>
+      <c r="B271" s="8" t="n"/>
+      <c r="C271" s="8" t="n"/>
+      <c r="D271" s="8" t="n"/>
+      <c r="E271" s="8" t="n"/>
+      <c r="F271" s="8" t="n"/>
+      <c r="G271" s="8" t="n"/>
+      <c r="H271" s="8" t="n"/>
+      <c r="I271" s="8" t="n"/>
+      <c r="J271" s="8" t="n"/>
+    </row>
+    <row r="272" ht="17" customHeight="1">
+      <c r="A272" s="8" t="n"/>
+      <c r="B272" s="8" t="n"/>
+      <c r="C272" s="8" t="n"/>
+      <c r="D272" s="8" t="n"/>
+      <c r="E272" s="8" t="n"/>
+      <c r="F272" s="8" t="n"/>
+      <c r="G272" s="8" t="n"/>
+      <c r="H272" s="8" t="n"/>
+      <c r="I272" s="8" t="n"/>
+      <c r="J272" s="8" t="n"/>
+    </row>
+    <row r="273" ht="17" customHeight="1">
+      <c r="A273" s="8" t="n"/>
+      <c r="B273" s="8" t="n"/>
+      <c r="C273" s="8" t="n"/>
+      <c r="D273" s="8" t="n"/>
+      <c r="E273" s="8" t="n"/>
+      <c r="F273" s="8" t="n"/>
+      <c r="G273" s="8" t="n"/>
+      <c r="H273" s="8" t="n"/>
+      <c r="I273" s="8" t="n"/>
+      <c r="J273" s="8" t="n"/>
+    </row>
+    <row r="274" ht="17" customHeight="1">
+      <c r="A274" s="8" t="n"/>
+      <c r="B274" s="8" t="n"/>
+      <c r="C274" s="8" t="n"/>
+      <c r="D274" s="8" t="n"/>
+      <c r="E274" s="8" t="n"/>
+      <c r="F274" s="8" t="n"/>
+      <c r="G274" s="8" t="n"/>
+      <c r="H274" s="8" t="n"/>
+      <c r="I274" s="8" t="n"/>
+      <c r="J274" s="8" t="n"/>
+    </row>
+    <row r="275" ht="17" customHeight="1">
+      <c r="A275" s="8" t="n"/>
+      <c r="B275" s="8" t="n"/>
+      <c r="C275" s="8" t="n"/>
+      <c r="D275" s="8" t="n"/>
+      <c r="E275" s="8" t="n"/>
+      <c r="F275" s="8" t="n"/>
+      <c r="G275" s="8" t="n"/>
+      <c r="H275" s="8" t="n"/>
+      <c r="I275" s="8" t="n"/>
+      <c r="J275" s="8" t="n"/>
+    </row>
+    <row r="276" ht="17" customHeight="1">
+      <c r="A276" s="8" t="n"/>
+      <c r="B276" s="8" t="n"/>
+      <c r="C276" s="8" t="n"/>
+      <c r="D276" s="8" t="n"/>
+      <c r="E276" s="8" t="n"/>
+      <c r="F276" s="8" t="n"/>
+      <c r="G276" s="8" t="n"/>
+      <c r="H276" s="8" t="n"/>
+      <c r="I276" s="8" t="n"/>
+      <c r="J276" s="8" t="n"/>
+    </row>
+    <row r="277" ht="17" customHeight="1">
+      <c r="A277" s="8" t="n"/>
+      <c r="B277" s="8" t="n"/>
+      <c r="C277" s="8" t="n"/>
+      <c r="D277" s="8" t="n"/>
+      <c r="E277" s="8" t="n"/>
+      <c r="F277" s="8" t="n"/>
+      <c r="G277" s="8" t="n"/>
+      <c r="H277" s="8" t="n"/>
+      <c r="I277" s="8" t="n"/>
+      <c r="J277" s="8" t="n"/>
+    </row>
+    <row r="278" ht="17" customHeight="1">
+      <c r="A278" s="8" t="n"/>
+      <c r="B278" s="8" t="n"/>
+      <c r="C278" s="8" t="n"/>
+      <c r="D278" s="8" t="n"/>
+      <c r="E278" s="8" t="n"/>
+      <c r="F278" s="8" t="n"/>
+      <c r="G278" s="8" t="n"/>
+      <c r="H278" s="8" t="n"/>
+      <c r="I278" s="8" t="n"/>
+      <c r="J278" s="8" t="n"/>
+    </row>
+    <row r="279" ht="17" customHeight="1">
+      <c r="A279" s="8" t="n"/>
+      <c r="B279" s="8" t="n"/>
+      <c r="C279" s="8" t="n"/>
+      <c r="D279" s="8" t="n"/>
+      <c r="E279" s="8" t="n"/>
+      <c r="F279" s="8" t="n"/>
+      <c r="G279" s="8" t="n"/>
+      <c r="H279" s="8" t="n"/>
+      <c r="I279" s="8" t="n"/>
+      <c r="J279" s="8" t="n"/>
+    </row>
+    <row r="280" ht="17" customHeight="1">
+      <c r="A280" s="8" t="n"/>
+      <c r="B280" s="8" t="n"/>
+      <c r="C280" s="8" t="n"/>
+      <c r="D280" s="8" t="n"/>
+      <c r="E280" s="8" t="n"/>
+      <c r="F280" s="8" t="n"/>
+      <c r="G280" s="8" t="n"/>
+      <c r="H280" s="8" t="n"/>
+      <c r="I280" s="8" t="n"/>
+      <c r="J280" s="8" t="n"/>
+    </row>
+    <row r="281" ht="17" customHeight="1">
+      <c r="A281" s="8" t="n"/>
+      <c r="B281" s="8" t="n"/>
+      <c r="C281" s="8" t="n"/>
+      <c r="D281" s="8" t="n"/>
+      <c r="E281" s="8" t="n"/>
+      <c r="F281" s="8" t="n"/>
+      <c r="G281" s="8" t="n"/>
+      <c r="H281" s="8" t="n"/>
+      <c r="I281" s="8" t="n"/>
+      <c r="J281" s="8" t="n"/>
+    </row>
+    <row r="282" ht="17" customHeight="1">
+      <c r="A282" s="8" t="n"/>
+      <c r="B282" s="8" t="n"/>
+      <c r="C282" s="8" t="n"/>
+      <c r="D282" s="8" t="n"/>
+      <c r="E282" s="8" t="n"/>
+      <c r="F282" s="8" t="n"/>
+      <c r="G282" s="8" t="n"/>
+      <c r="H282" s="8" t="n"/>
+      <c r="I282" s="8" t="n"/>
+      <c r="J282" s="8" t="n"/>
+    </row>
+    <row r="283" ht="17" customHeight="1">
+      <c r="A283" s="8" t="n"/>
+      <c r="B283" s="8" t="n"/>
+      <c r="C283" s="8" t="n"/>
+      <c r="D283" s="8" t="n"/>
+      <c r="E283" s="8" t="n"/>
+      <c r="F283" s="8" t="n"/>
+      <c r="G283" s="8" t="n"/>
+      <c r="H283" s="8" t="n"/>
+      <c r="I283" s="8" t="n"/>
+      <c r="J283" s="8" t="n"/>
+    </row>
+    <row r="284" ht="17" customHeight="1">
+      <c r="A284" s="8" t="n"/>
+      <c r="B284" s="8" t="n"/>
+      <c r="C284" s="8" t="n"/>
+      <c r="D284" s="8" t="n"/>
+      <c r="E284" s="8" t="n"/>
+      <c r="F284" s="8" t="n"/>
+      <c r="G284" s="8" t="n"/>
+      <c r="H284" s="8" t="n"/>
+      <c r="I284" s="8" t="n"/>
+      <c r="J284" s="8" t="n"/>
+    </row>
+    <row r="285" ht="17" customHeight="1">
+      <c r="A285" s="8" t="n"/>
+      <c r="B285" s="8" t="n"/>
+      <c r="C285" s="8" t="n"/>
+      <c r="D285" s="8" t="n"/>
+      <c r="E285" s="8" t="n"/>
+      <c r="F285" s="8" t="n"/>
+      <c r="G285" s="8" t="n"/>
+      <c r="H285" s="8" t="n"/>
+      <c r="I285" s="8" t="n"/>
+      <c r="J285" s="8" t="n"/>
+    </row>
+    <row r="286" ht="17" customHeight="1">
+      <c r="A286" s="8" t="n"/>
+      <c r="B286" s="8" t="n"/>
+      <c r="C286" s="8" t="n"/>
+      <c r="D286" s="8" t="n"/>
+      <c r="E286" s="8" t="n"/>
+      <c r="F286" s="8" t="n"/>
+      <c r="G286" s="8" t="n"/>
+      <c r="H286" s="8" t="n"/>
+      <c r="I286" s="8" t="n"/>
+      <c r="J286" s="8" t="n"/>
+    </row>
+    <row r="287" ht="17" customHeight="1">
+      <c r="A287" s="8" t="n"/>
+      <c r="B287" s="8" t="n"/>
+      <c r="C287" s="8" t="n"/>
+      <c r="D287" s="8" t="n"/>
+      <c r="E287" s="8" t="n"/>
+      <c r="F287" s="8" t="n"/>
+      <c r="G287" s="8" t="n"/>
+      <c r="H287" s="8" t="n"/>
+      <c r="I287" s="8" t="n"/>
+      <c r="J287" s="8" t="n"/>
+    </row>
+    <row r="288" ht="17" customHeight="1">
+      <c r="A288" s="8" t="n"/>
+      <c r="B288" s="8" t="n"/>
+      <c r="C288" s="8" t="n"/>
+      <c r="D288" s="8" t="n"/>
+      <c r="E288" s="8" t="n"/>
+      <c r="F288" s="8" t="n"/>
+      <c r="G288" s="8" t="n"/>
+      <c r="H288" s="8" t="n"/>
+      <c r="I288" s="8" t="n"/>
+      <c r="J288" s="8" t="n"/>
+    </row>
+    <row r="289" ht="17" customHeight="1">
+      <c r="A289" s="8" t="n"/>
+      <c r="B289" s="8" t="n"/>
+      <c r="C289" s="8" t="n"/>
+      <c r="D289" s="8" t="n"/>
+      <c r="E289" s="8" t="n"/>
+      <c r="F289" s="8" t="n"/>
+      <c r="G289" s="8" t="n"/>
+      <c r="H289" s="8" t="n"/>
+      <c r="I289" s="8" t="n"/>
+      <c r="J289" s="8" t="n"/>
+    </row>
+    <row r="290" ht="17" customHeight="1">
+      <c r="A290" s="8" t="n"/>
+      <c r="B290" s="8" t="n"/>
+      <c r="C290" s="8" t="n"/>
+      <c r="D290" s="8" t="n"/>
+      <c r="E290" s="8" t="n"/>
+      <c r="F290" s="8" t="n"/>
+      <c r="G290" s="8" t="n"/>
+      <c r="H290" s="8" t="n"/>
+      <c r="I290" s="8" t="n"/>
+      <c r="J290" s="8" t="n"/>
+    </row>
+    <row r="291" ht="17" customHeight="1">
+      <c r="A291" s="8" t="n"/>
+      <c r="B291" s="8" t="n"/>
+      <c r="C291" s="8" t="n"/>
+      <c r="D291" s="8" t="n"/>
+      <c r="E291" s="8" t="n"/>
+      <c r="F291" s="8" t="n"/>
+      <c r="G291" s="8" t="n"/>
+      <c r="H291" s="8" t="n"/>
+      <c r="I291" s="8" t="n"/>
+      <c r="J291" s="8" t="n"/>
+    </row>
+    <row r="292" ht="17" customHeight="1">
+      <c r="A292" s="8" t="n"/>
+      <c r="B292" s="8" t="n"/>
+      <c r="C292" s="8" t="n"/>
+      <c r="D292" s="8" t="n"/>
+      <c r="E292" s="8" t="n"/>
+      <c r="F292" s="8" t="n"/>
+      <c r="G292" s="8" t="n"/>
+      <c r="H292" s="8" t="n"/>
+      <c r="I292" s="8" t="n"/>
+      <c r="J292" s="8" t="n"/>
+    </row>
+    <row r="293" ht="17" customHeight="1">
+      <c r="A293" s="8" t="n"/>
+      <c r="B293" s="8" t="n"/>
+      <c r="C293" s="8" t="n"/>
+      <c r="D293" s="8" t="n"/>
+      <c r="E293" s="8" t="n"/>
+      <c r="F293" s="8" t="n"/>
+      <c r="G293" s="8" t="n"/>
+      <c r="H293" s="8" t="n"/>
+      <c r="I293" s="8" t="n"/>
+      <c r="J293" s="8" t="n"/>
+    </row>
+    <row r="294" ht="17" customHeight="1">
+      <c r="A294" s="8" t="n"/>
+      <c r="B294" s="8" t="n"/>
+      <c r="C294" s="8" t="n"/>
+      <c r="D294" s="8" t="n"/>
+      <c r="E294" s="8" t="n"/>
+      <c r="F294" s="8" t="n"/>
+      <c r="G294" s="8" t="n"/>
+      <c r="H294" s="8" t="n"/>
+      <c r="I294" s="8" t="n"/>
+      <c r="J294" s="8" t="n"/>
+    </row>
+    <row r="295" ht="17" customHeight="1">
+      <c r="A295" s="8" t="n"/>
+      <c r="B295" s="8" t="n"/>
+      <c r="C295" s="8" t="n"/>
+      <c r="D295" s="8" t="n"/>
+      <c r="E295" s="8" t="n"/>
+      <c r="F295" s="8" t="n"/>
+      <c r="G295" s="8" t="n"/>
+      <c r="H295" s="8" t="n"/>
+      <c r="I295" s="8" t="n"/>
+      <c r="J295" s="8" t="n"/>
+    </row>
+    <row r="296" ht="17" customHeight="1">
+      <c r="A296" s="8" t="n"/>
+      <c r="B296" s="8" t="n"/>
+      <c r="C296" s="8" t="n"/>
+      <c r="D296" s="8" t="n"/>
+      <c r="E296" s="8" t="n"/>
+      <c r="F296" s="8" t="n"/>
+      <c r="G296" s="8" t="n"/>
+      <c r="H296" s="8" t="n"/>
+      <c r="I296" s="8" t="n"/>
+      <c r="J296" s="8" t="n"/>
+    </row>
+    <row r="297" ht="17" customHeight="1">
+      <c r="A297" s="8" t="n"/>
+      <c r="B297" s="8" t="n"/>
+      <c r="C297" s="8" t="n"/>
+      <c r="D297" s="8" t="n"/>
+      <c r="E297" s="8" t="n"/>
+      <c r="F297" s="8" t="n"/>
+      <c r="G297" s="8" t="n"/>
+      <c r="H297" s="8" t="n"/>
+      <c r="I297" s="8" t="n"/>
+      <c r="J297" s="8" t="n"/>
+    </row>
+    <row r="298" ht="17" customHeight="1">
+      <c r="A298" s="8" t="n"/>
+      <c r="B298" s="8" t="n"/>
+      <c r="C298" s="8" t="n"/>
+      <c r="D298" s="8" t="n"/>
+      <c r="E298" s="8" t="n"/>
+      <c r="F298" s="8" t="n"/>
+      <c r="G298" s="8" t="n"/>
+      <c r="H298" s="8" t="n"/>
+      <c r="I298" s="8" t="n"/>
+      <c r="J298" s="8" t="n"/>
+    </row>
+    <row r="299" ht="17" customHeight="1">
+      <c r="A299" s="8" t="n"/>
+      <c r="B299" s="8" t="n"/>
+      <c r="C299" s="8" t="n"/>
+      <c r="D299" s="8" t="n"/>
+      <c r="E299" s="8" t="n"/>
+      <c r="F299" s="8" t="n"/>
+      <c r="G299" s="8" t="n"/>
+      <c r="H299" s="8" t="n"/>
+      <c r="I299" s="8" t="n"/>
+      <c r="J299" s="8" t="n"/>
+    </row>
+    <row r="300" ht="17" customHeight="1">
+      <c r="A300" s="8" t="n"/>
+      <c r="B300" s="8" t="n"/>
+      <c r="C300" s="8" t="n"/>
+      <c r="D300" s="8" t="n"/>
+      <c r="E300" s="8" t="n"/>
+      <c r="F300" s="8" t="n"/>
+      <c r="G300" s="8" t="n"/>
+      <c r="H300" s="8" t="n"/>
+      <c r="I300" s="8" t="n"/>
+      <c r="J300" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="C6:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ASSET,LIABILITY,INCOME,EXPENSE,EQUITY"</formula1>
+  <dataValidations count="5">
+    <dataValidation sqref="C6:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'_Lookups'!$A$1:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="F6:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
+    <dataValidation sqref="D6:D300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'_Lookups'!$B$1:$B$12</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"DR,CR"</formula1>
+    <dataValidation sqref="F6:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'_Lookups'!$C$1:$C$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="G6:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'_Lookups'!$C$1:$C$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="I6:I300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'_Lookups'!$D$1:$D$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3134,7 +4341,150 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ASSET</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Current Asset</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>DR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LIABILITY</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fixed Asset</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>INCOME</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Current Liability</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EXPENSE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Long-term Liability</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Operating Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Salaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Administrative</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Opening Balance</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -3143,7 +4493,7 @@
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>SmartAppt – COA Upload Instructions</t>
+          <t>SmartAppt – Chart of Accounts Upload Template</t>
         </is>
       </c>
     </row>
@@ -3151,159 +4501,166 @@
       <c r="A2" s="10" t="inlineStr"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>1.  Fill in the 'Chart of Accounts' sheet starting from Row 6.</t>
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>STEPS</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>2.  Rows 1–5 are header/example rows — do not delete them.</t>
+          <t>1. Fill in the 'Chart of Accounts' sheet starting from Row 6.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>3.  Use the dropdown cells for Type, Is Group?, Is Control Account?, OB Side.</t>
+          <t>2. Rows 1–5 are header/example rows — do not delete or edit them.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>4.  Opening balance fields are optional. Leave blank if not applicable.</t>
+          <t>3. Use the dropdown menus for: Type, Sub-type, Is Group?, Is Control Account?, OB Side.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    - 'Opening Balance' must be a number without commas or currency symbols.</t>
+          <t>4. Opening balance fields are optional. Leave blank if not needed.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    - 'OB Side' is DR (debit) or CR (credit).</t>
+          <t xml:space="preserve">   - 'Opening Balance' must be a number with no commas or currency symbol.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    - 'OB As-on Date' must be in YYYY-MM-DD format (e.g. 2025-03-31).</t>
+          <t xml:space="preserve">   - 'OB Side' is DR (Debit) or CR (Credit).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>5.  Control accounts (Is Control Account? = Yes): set Opening Balance on the</t>
+          <t xml:space="preserve">   - 'OB As-on Date' must be YYYY-MM-DD format (e.g. 2025-03-31).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Business Partner record, NOT here. Leave OB fields blank for control accounts.</t>
+          <t>5. Control accounts (Is Control Account? = Yes): leave OB fields blank.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>6.  Account codes must be unique. Duplicate codes are skipped on import.</t>
+          <t xml:space="preserve">   Opening balance for control accounts is set on each Business Partner record.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>7.  Save the file as .xlsx and upload via Chart of Accounts → Upload Accounts.</t>
+          <t>6. Account codes must be unique. Codes already in the system are skipped on import.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>7. Save as .xlsx and upload via: Chart of Accounts → Upload Accounts.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Column Reference:</t>
-        </is>
-      </c>
+      <c r="A15" s="10" t="inlineStr"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  code                  Unique account code (e.g. 1006)</t>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>COLUMN REFERENCE</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  name                  Account name</t>
+          <t xml:space="preserve">  code                   Unique account code (e.g. 1006)  [Required]</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  type                  ASSET | LIABILITY | INCOME | EXPENSE | EQUITY</t>
+          <t xml:space="preserve">  name                   Account name  [Required]</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  sub_type              e.g. Current Asset, Utility, Salaries (optional)</t>
+          <t xml:space="preserve">  type                   ASSET | LIABILITY | INCOME | EXPENSE | EQUITY  [Required]</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  description           Short description (optional)</t>
+          <t xml:space="preserve">  sub_type               e.g. Current Asset, Utility, Salaries  [Optional]</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  is_group              Yes or No</t>
+          <t xml:space="preserve">  description            Short description  [Optional]</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  is_control_account    Yes or No</t>
+          <t xml:space="preserve">  is_group               Yes or No  [Optional, default: No]</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  opening_balance       Numeric amount (optional)</t>
+          <t xml:space="preserve">  is_control_account     Yes or No  [Optional, default: No]</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  opening_balance_type  DR or CR</t>
+          <t xml:space="preserve">  opening_balance        Numeric amount  [Optional]</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  opening_balance_date  YYYY-MM-DD (optional)</t>
+          <t xml:space="preserve">  opening_balance_type   DR or CR  [Optional]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  opening_balance_date   YYYY-MM-DD  [Optional]</t>
         </is>
       </c>
     </row>

</xml_diff>